<commit_message>
Refine table profile generation and skill docs
</commit_message>
<xml_diff>
--- a/res/task.xlsx
+++ b/res/task.xlsx
@@ -3769,7 +3769,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{984B885C-48D0-4D9B-AAB3-39C5F463E278}">
-  <dimension ref="A1:E10"/>
+  <dimension ref="A1:E11"/>
   <sheetFormatPr defaultColWidth="8.875" defaultRowHeight="14.25" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="9" style="39"/>
@@ -3933,6 +3933,31 @@
       </c>
       <c r="E10" t="s">
         <v>244</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>GATE_SIEGE_START_TIME</t>
+        </is>
+      </c>
+      <c r="C11">
+        <v>1000</v>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>int</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>开始攻城时间</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>